<commit_message>
release v2.9.1 bilingual travel scope package
</commit_message>
<xml_diff>
--- a/examples/demo/Demo China Trip旅行攻略大全-en.xlsx
+++ b/examples/demo/Demo China Trip旅行攻略大全-en.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>7 days</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -623,12 +623,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>演示住宿</t>
+          <t>演示住宿一</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Demo Hotel</t>
+          <t>Demo Hotel One</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -645,7 +645,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>美食</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -655,29 +655,29 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>演示餐厅</t>
+          <t>演示住宿二</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Demo Restaurant</t>
+          <t>Demo Hotel Two</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>39.9050,116.4080</t>
+          <t>39.9060,116.4100</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=39.905,116.408</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.906,116.41</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>景点</t>
+          <t>美食</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -687,29 +687,29 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>演示景点</t>
+          <t>演示餐厅一</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Demo Attraction</t>
+          <t>Demo Restaurant One</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>39.9048,116.4077</t>
+          <t>39.9050,116.4080</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=39.9048,116.4077</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.905,116.408</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>交通-出发</t>
+          <t>美食</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -719,44 +719,236 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>演示城市</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
+          <t>演示餐厅二</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Demo Restaurant Two</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>39.9042,116.4074</t>
+          <t>39.9070,116.4120</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=39.9042,116.4074</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.907,116.412</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>演示景点一</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction One</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>39.9048,116.4077</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.9048,116.4077</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>演示景点二</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction Two</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>39.9055,116.4090</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.9055,116.409</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>演示景点三</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction Three</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>39.9065,116.4110</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.9065,116.411</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>演示景点四</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction Four</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>39.9080,116.4130</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.908,116.413</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>演示景点五</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction Five</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>39.9090,116.4140</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.909,116.414</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>交通-出发</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>39.9042,116.4074</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=39.9042,116.4074</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>交通-到达</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>演示城市</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>演示城市</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>39.9050,116.4080</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=39.905,116.408</t>
         </is>
@@ -773,7 +965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -837,7 +1029,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>演示景点</t>
+          <t>演示景点一</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -867,7 +1059,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>演示餐厅</t>
+          <t>演示餐厅一</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -884,23 +1076,353 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Day 1</t>
+          <t>Day 2</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>演示景点二</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>39.9055,116.4090</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>酒店</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>演示住宿</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>演示住宿一</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>39.9042,116.4074</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>演示城市→演示城市</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>39.9042,116.4074</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>演示景点三</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>39.9065,116.4110</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Day 4</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>餐厅</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>演示餐厅二</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>39.9070,116.4120</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Day 4</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>演示景点四</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>39.9080,116.4130</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Day 5</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>演示景点五</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>39.9090,116.4140</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Day 5</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>酒店</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>演示住宿二</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>39.9060,116.4100</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Day 6</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>演示景点一</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>39.9048,116.4077</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Day 6</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>餐厅</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>演示餐厅二</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>39.9070,116.4120</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Day 7</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>演示景点二</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>39.9055,116.4090</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Demo Route</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Day 7</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>酒店</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>演示住宿一</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>39.9042,116.4074</t>
         </is>
@@ -974,7 +1496,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>7 days</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -984,7 +1506,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Shows the output pipeline</t>
+          <t>Shows a complete multi-day output pipeline</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1014,7 +1536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1185,12 +1707,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>演示住宿</t>
+          <t>演示住宿一</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Demo Hotel</t>
+          <t>Demo Hotel One</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1218,9 +1740,74 @@
           <t>39.9042,116.4074</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-hotel-one-1.jpg</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-hotel-one-2.jpg</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic fixture record</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>演示住宿二</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Demo Hotel Two</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Demo accommodation</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Demo:4.2</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>39.9060,116.4100</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-hotel-two-1.jpg</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-hotel-two-2.jpg</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Synthetic fixture record</t>
         </is>
@@ -1237,7 +1824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1408,12 +1995,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>演示餐厅</t>
+          <t>演示餐厅一</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Demo Restaurant</t>
+          <t>Demo Restaurant One</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1428,7 +2015,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Demo:4.0</t>
+          <t>Demo:4.1</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1441,11 +2028,76 @@
           <t>39.9050,116.4080</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-restaurant-one-1.jpg</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-restaurant-one-2.jpg</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Synthetic fixture address</t>
+          <t>Synthetic fixture record</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>演示餐厅二</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Demo Restaurant Two</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Demo cuisine</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Demo:4.3</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>39.9070,116.4120</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-restaurant-two-1.jpg</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-restaurant-two-2.jpg</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic fixture record</t>
         </is>
       </c>
     </row>
@@ -1579,7 +2231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1750,12 +2402,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>演示景点</t>
+          <t>演示景点一</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Demo Attraction</t>
+          <t>Demo Attraction One</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1778,14 +2430,250 @@
           <t>39.9048,116.4077</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-one-1.jpg</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-one-2.jpg</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>1 hour</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic fixture description</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>演示景点二</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction Two</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Demo attraction</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Demo:4.1</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>39.9055,116.4090</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-two-1.jpg</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-two-2.jpg</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2 hours</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic fixture description</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>演示景点三</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction Three</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Demo attraction</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Demo:4.2</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>39.9065,116.4110</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-three-1.jpg</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-three-2.jpg</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2 hours</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic fixture description</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>演示景点四</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction Four</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Demo attraction</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Demo:4.3</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>39.9080,116.4130</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-four-1.jpg</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-four-2.jpg</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>1 hour</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic fixture description</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>演示城市</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>演示景点五</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Demo Attraction Five</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Demo attraction</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Demo:4.4</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>39.9090,116.4140</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-five-1.jpg</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/demo-attraction-five-2.jpg</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2 hours</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Synthetic fixture description</t>
         </is>
@@ -1886,7 +2774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1985,41 +2873,251 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Demo date</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Demo itinerary</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Demo date</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Demo itinerary</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Day 4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Demo date</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Demo itinerary</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Day 5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Demo date</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Demo itinerary</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Day 6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Demo date</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Demo itinerary</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Day 7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Demo date</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Demo itinerary</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>2 days</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>7 days</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Demo total</t>
         </is>
       </c>
-      <c r="D3" s="2">
-        <f>SUM(D2:D2)</f>
+      <c r="D9" s="2">
+        <f>SUM(D2:D8)</f>
         <v/>
       </c>
-      <c r="E3" s="2">
-        <f>SUM(E2:E2)</f>
+      <c r="E9" s="2">
+        <f>SUM(E2:E8)</f>
         <v/>
       </c>
-      <c r="F3" s="2">
-        <f>SUM(F2:F2)</f>
+      <c r="F9" s="2">
+        <f>SUM(F2:F8)</f>
         <v/>
       </c>
-      <c r="G3" s="2">
-        <f>SUM(G2:G2)</f>
+      <c r="G9" s="2">
+        <f>SUM(G2:G8)</f>
         <v/>
       </c>
-      <c r="H3" s="2">
-        <f>SUM(H2:H2)</f>
+      <c r="H9" s="2">
+        <f>SUM(H2:H8)</f>
         <v/>
       </c>
-      <c r="I3" s="2">
-        <f>SUM(I2:I2)</f>
+      <c r="I9" s="2">
+        <f>SUM(I2:I8)</f>
         <v/>
       </c>
     </row>
@@ -2097,7 +3195,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CN/EN output can be generated from the same fixture.</t>
+          <t>CN/EN output is generated from the same fixture.</t>
         </is>
       </c>
     </row>

</xml_diff>